<commit_message>
S-013: close the gate (Evidence + CLAUDE.md + tracker + OQ-001 note)
Records GREEN verdict on S-013 with two explicit deferrals (live CI, second-
machine clean-clone smoke) and OQ-001 left Open (deferred). All 13 packets now
GREEN; product gate (D4 §5) met.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project_Progress_Tracker.xlsx
+++ b/Project_Progress_Tracker.xlsx
@@ -3075,17 +3075,17 @@
       </c>
       <c r="H17" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I17" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K17" s="17" t="inlineStr">
@@ -3100,7 +3100,7 @@
       </c>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>Pre-build files authored. Final gate; includes clean-clone smoke (NFR Q-008).</t>
+          <t>GREEN with deferrals. README + CI workflow + git init + initial commit (3dcb799). AC3 (live CI) and AC5 (clean-clone smoke on second machine) explicitly deferred per user direction; OQ-001 stays Open (deferred). All 6 ACs structurally met; see Evidence.md §Deferrals.</t>
         </is>
       </c>
     </row>
@@ -5815,10 +5815,14 @@
       </c>
       <c r="E93" s="17" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="F93" s="17" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F93" s="17" t="inlineStr">
+        <is>
+          <t>README.md §Quickstart copy-pasteable; commands derived from the working tree that already produces 37+35 green tests.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="18" t="inlineStr">
@@ -5843,10 +5847,14 @@
       </c>
       <c r="E94" s="18" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="F94" s="18" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F94" s="18" t="inlineStr">
+        <is>
+          <t>backend/.env.example + frontend/.env.example complete; .env files not staged (git ls-files | grep .env$ empty).</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="17" t="inlineStr">
@@ -5871,10 +5879,14 @@
       </c>
       <c r="E95" s="17" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="F95" s="17" t="inlineStr"/>
+          <t>Pass (structure) / deferred (live)</t>
+        </is>
+      </c>
+      <c r="F95" s="17" t="inlineStr">
+        <is>
+          <t>.github/workflows/ci.yml created per D4 §6; will run on first push to a GitHub remote (not yet pushed).</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="18" t="inlineStr">
@@ -5899,10 +5911,14 @@
       </c>
       <c r="E96" s="18" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="F96" s="18" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F96" s="18" t="inlineStr">
+        <is>
+          <t>README §Deploy covers Render service config + Vercel project config; labelled illustrative because OQ-001 is deferred.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="17" t="inlineStr">
@@ -5927,10 +5943,14 @@
       </c>
       <c r="E97" s="17" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="F97" s="17" t="inlineStr"/>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="F97" s="17" t="inlineStr">
+        <is>
+          <t>Per user direction (2026-06-29). To close: run README §Quickstart on a fresh machine with stopwatch + screenshot, append §AC5 Live Smoke block to Evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="18" t="inlineStr">
@@ -5955,10 +5975,14 @@
       </c>
       <c r="E98" s="18" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="F98" s="18" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F98" s="18" t="inlineStr">
+        <is>
+          <t>Verified post-commit on 3dcb799: empty. Also verified .venv, node_modules, __pycache__, dist all unstaged.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -6067,7 +6091,7 @@
       </c>
       <c r="C5" s="17" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open (deferred)</t>
         </is>
       </c>
       <c r="D5" s="17" t="inlineStr">
@@ -6077,7 +6101,7 @@
       </c>
       <c r="E5" s="17" t="inlineStr">
         <is>
-          <t>TBD before S-013</t>
+          <t>Deferred past S-013 close at user direction (2026-06-29). README §Deploy documents Render + Vercel illustratively.</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
@@ -6087,7 +6111,7 @@
       </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S-013: close AC3 (live CI verified)
PR #1 run 28359504205 (pull_request) and post-merge run 28359606351 (push to
main) both green across backend, frontend, security jobs. Flips AC3 from
"deferred (live)" to "Pass" in Evidence, tracker, and CLAUDE.md.

Remaining S-013 deferrals: AC5 (second-machine clean-clone smoke) and OQ-001
(deploy target choice).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project_Progress_Tracker.xlsx
+++ b/Project_Progress_Tracker.xlsx
@@ -3100,7 +3100,7 @@
       </c>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>GREEN with deferrals. README + CI workflow + git init + initial commit (3dcb799). AC3 (live CI) and AC5 (clean-clone smoke on second machine) explicitly deferred per user direction; OQ-001 stays Open (deferred). All 6 ACs structurally met; see Evidence.md §Deferrals.</t>
+          <t>GREEN. AC3 live-verified 2026-06-29 (PR #1 + post-merge push, both green). AC5 (second-machine smoke) and OQ-001 (deploy target) remain deferred per Evidence.md §Deferrals.</t>
         </is>
       </c>
     </row>
@@ -5879,12 +5879,12 @@
       </c>
       <c r="E95" s="17" t="inlineStr">
         <is>
-          <t>Pass (structure) / deferred (live)</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="F95" s="17" t="inlineStr">
         <is>
-          <t>.github/workflows/ci.yml created per D4 §6; will run on first push to a GitHub remote (not yet pushed).</t>
+          <t>Live-verified 2026-06-29: PR #1 run 28359504205 green (41s); post-merge push-to-main run 28359606351 green (34s). Both trigger paths confirmed.</t>
         </is>
       </c>
     </row>

</xml_diff>